<commit_message>
Forzar version actual con Excel actualizado
</commit_message>
<xml_diff>
--- a/DRIVE TRHU BASE.xlsx
+++ b/DRIVE TRHU BASE.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="8910" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="8910"/>
   </bookViews>
   <sheets>
     <sheet name="Drive HME" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1621" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1631" uniqueCount="246">
   <si>
     <t>N°</t>
   </si>
@@ -760,6 +760,9 @@
   </si>
   <si>
     <t xml:space="preserve">cambio de cargador de baterias </t>
+  </si>
+  <si>
+    <t>STB134</t>
   </si>
 </sst>
 </file>
@@ -1443,7 +1446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z12"/>
+  <dimension ref="A1:Z13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -2405,6 +2408,86 @@
       </c>
       <c r="Y12" s="31"/>
       <c r="Z12" s="31" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" s="32" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="29">
+        <v>12</v>
+      </c>
+      <c r="B13" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="29" t="s">
+        <v>245</v>
+      </c>
+      <c r="D13" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" s="30">
+        <v>4</v>
+      </c>
+      <c r="F13" s="30">
+        <v>2</v>
+      </c>
+      <c r="G13" s="30">
+        <f t="shared" ref="G13" si="2">E13+F13</f>
+        <v>6</v>
+      </c>
+      <c r="H13" s="30">
+        <v>1</v>
+      </c>
+      <c r="I13" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="J13" s="31">
+        <v>7</v>
+      </c>
+      <c r="K13" s="31">
+        <v>1</v>
+      </c>
+      <c r="L13" s="31">
+        <f t="shared" ref="L13" si="3">J13+K13</f>
+        <v>8</v>
+      </c>
+      <c r="M13" s="30">
+        <v>1</v>
+      </c>
+      <c r="N13" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="O13" s="30">
+        <v>1</v>
+      </c>
+      <c r="P13" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q13" s="30">
+        <v>1</v>
+      </c>
+      <c r="R13" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="S13" s="30">
+        <v>4</v>
+      </c>
+      <c r="T13" s="30">
+        <v>1</v>
+      </c>
+      <c r="U13" s="30">
+        <v>1</v>
+      </c>
+      <c r="V13" s="30">
+        <v>1</v>
+      </c>
+      <c r="W13" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="X13" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y13" s="31"/>
+      <c r="Z13" s="31" t="s">
         <v>58</v>
       </c>
     </row>

</xml_diff>